<commit_message>
Simplify opportunities tracking to tracker.xlsx and drop legacy builders.
Rename the working shortlist to tracker.xlsx, remove build_opportunities.py and the peri-urban stub, and point the SoT, folder layout, and new-scan script at the new paths.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/opportunities/new_opportunities.xlsx
+++ b/opportunities/new_opportunities.xlsx
@@ -927,7 +927,7 @@
       </c>
       <c r="B2" s="11" t="inlineStr">
         <is>
-          <t>2026-07-29 12:51</t>
+          <t>2026-07-29 12:56</t>
         </is>
       </c>
     </row>
@@ -939,7 +939,7 @@
       </c>
       <c r="B3" s="11" t="inlineStr">
         <is>
-          <t>CLEARED and rebuilt new_opportunities.xlsx (29 July 2026). Fresh open-call scan only. Does not replace best_opportinities.xlsx. Deduped against working tracker and build_opportunities.py titles.</t>
+          <t>CLEARED and rebuilt new_opportunities.xlsx (29 July 2026). Fresh open-call scan only. Does not replace tracker.xlsx. Deduped against the working tracker.</t>
         </is>
       </c>
     </row>
@@ -1042,12 +1042,12 @@
     <row r="12" ht="70" customHeight="1">
       <c r="A12" s="11" t="inlineStr">
         <is>
-          <t>Excluded (already on best / canonical tracker)</t>
+          <t>Excluded (already on working tracker)</t>
         </is>
       </c>
       <c r="B12" s="11" t="inlineStr">
         <is>
-          <t>AWIEF; Africa Health-Tech Accelerator; Nexa PoC (submitted); DPI Safeguards (submitted); DoS Uganda MOU; Japan GGP; Jay Shetty; Yunus; ANeSA LoI; FID reopen watch; DIV; Gadfly; WHS Youth Group; SIARP; Brandtech; AES Fellowship; and other build_opportunities.py titles.</t>
+          <t>AWIEF; Africa Health-Tech Accelerator; Nexa PoC (submitted); DPI Safeguards (submitted); DoS Uganda MOU; Japan GGP; Jay Shetty; Yunus; ANeSA LoI; FID reopen watch; DIV; Gadfly; WHS Youth Group; SIARP; Brandtech; AES Fellowship; and other titles already listed in tracker.xlsx.</t>
         </is>
       </c>
     </row>
@@ -1107,7 +1107,7 @@
       </c>
       <c r="B17" s="11" t="inlineStr">
         <is>
-          <t>opportunities/best_opportinities.xlsx</t>
+          <t>opportunities/tracker.xlsx</t>
         </is>
       </c>
     </row>

</xml_diff>